<commit_message>
Added WindowsDamage.pdf (our own document) and the corresponding changes to other docs,
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA94DCD-F68B-014F-9DB0-6B1C97AEE748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64115B25-C962-1941-9B17-80836A94987F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="47900" yWindow="1320" windowWidth="22020" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="660" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Window Estimate" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="126">
   <si>
     <t>Pella Window &amp; Door Replacement Estimate</t>
   </si>
@@ -107,19 +107,10 @@
     <t>Pella Reserve, Traditional Casement Right, 22 X 58, White</t>
   </si>
   <si>
-    <t>Master W-383</t>
-  </si>
-  <si>
     <t>Pella Reserve, Traditional Casement Left, 22 X 60, White</t>
   </si>
   <si>
-    <t>Master W-384</t>
-  </si>
-  <si>
     <t>Pella Reserve, Traditional Sash Set, Fixed, 54 X 60, White</t>
-  </si>
-  <si>
-    <t>Master W-385</t>
   </si>
   <si>
     <t>Pella Reserve, Traditional Casement Right, 22 X 60, White</t>
@@ -237,9 +228,6 @@
 (upper south-east facing)</t>
   </si>
   <si>
-    <t>A-121, A-122-123</t>
-  </si>
-  <si>
     <t>Family W 231-233
 (3 sashes upper  window)</t>
   </si>
@@ -248,9 +236,6 @@
 (3-sashes, main window)</t>
   </si>
   <si>
-    <t>A-115, A--6, A-117</t>
-  </si>
-  <si>
     <t>Family W 230
 (Lower south-east facing)</t>
   </si>
@@ -265,9 +250,6 @@
 (North-east facing, upper)</t>
   </si>
   <si>
-    <t>A-134, A-135</t>
-  </si>
-  <si>
     <t>Missing</t>
   </si>
   <si>
@@ -275,12 +257,6 @@
 (North-east facing, Lower)</t>
   </si>
   <si>
-    <t>A-126, A-127, A-128</t>
-  </si>
-  <si>
-    <t>A-139, A-140</t>
-  </si>
-  <si>
     <t>A-141</t>
   </si>
   <si>
@@ -288,13 +264,7 @@
 (South-East facing by sliding door)</t>
   </si>
   <si>
-    <t>A-148 (trim), A-149,  2.4.6</t>
-  </si>
-  <si>
     <t>2.4.1, A-153, A-156</t>
-  </si>
-  <si>
-    <t>A-158</t>
   </si>
   <si>
     <t>A-162, A-163</t>
@@ -343,9 +313,6 @@
     <t>A-179, 2.3.5</t>
   </si>
   <si>
-    <t>A-183, 2.3.6</t>
-  </si>
-  <si>
     <t>Bedroom 3 W-388-390
 (Bedroom above office)</t>
   </si>
@@ -353,9 +320,6 @@
     <t>2.7.1, 2.7.2</t>
   </si>
   <si>
-    <t>A-200, 2.6.1</t>
-  </si>
-  <si>
     <t>Bedroom 5 W 11-113
 (Below office)</t>
   </si>
@@ -401,10 +365,6 @@
     <t>Appraisal award</t>
   </si>
   <si>
-    <t>W 247-248
-(Kitchen east facung(</t>
-  </si>
-  <si>
     <t>W 249-250
 (Kitchen east facung(</t>
   </si>
@@ -416,6 +376,74 @@
   </si>
   <si>
     <t>Sales Tax @ 8.525%:</t>
+  </si>
+  <si>
+    <t>Dents in Report</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>FromPhoto</t>
+  </si>
+  <si>
+    <t>A-119, A-121, A-122-123
+2.1.4, 2.1.5, 2.1.6</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>A-115, A--116, A-117
+2.1.11</t>
+  </si>
+  <si>
+    <t>A-134, A-135
+2.1.9</t>
+  </si>
+  <si>
+    <t>A-126, A-127, A-128
+2.1.8</t>
+  </si>
+  <si>
+    <t>Master W-383 (south-east)</t>
+  </si>
+  <si>
+    <t>A-148 (trim), A-151, A-149,  2.4.6</t>
+  </si>
+  <si>
+    <t>Master W-384 (center, east)</t>
+  </si>
+  <si>
+    <t>Master W-385 (North-east)</t>
+  </si>
+  <si>
+    <t>A-158, 2.4.3</t>
+  </si>
+  <si>
+    <t>A-139, A-140, 2.2.1</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t>2.3.2, A-170</t>
+  </si>
+  <si>
+    <t>2.3.6</t>
+  </si>
+  <si>
+    <t>2.6.1</t>
+  </si>
+  <si>
+    <t>????</t>
+  </si>
+  <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>W 247-248
+(Kitchen east facing)</t>
   </si>
 </sst>
 </file>
@@ -550,7 +578,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -617,34 +645,36 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -909,7 +939,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -917,36 +947,36 @@
     <col min="3" max="3" width="62" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="24.5" customWidth="1"/>
+    <col min="6" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -966,15 +996,18 @@
         <v>10</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>10</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>11</v>
@@ -989,14 +1022,15 @@
         <f t="shared" ref="F8:F45" si="0">D8*E8</f>
         <v>4480.9799999999996</v>
       </c>
-      <c r="G8" s="24"/>
-    </row>
-    <row r="9" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G8" s="20"/>
+      <c r="H8" s="24"/>
+    </row>
+    <row r="9" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>15</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>12</v>
@@ -1011,11 +1045,14 @@
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G9" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>20</v>
       </c>
@@ -1035,16 +1072,19 @@
         <f t="shared" si="0"/>
         <v>7085.76</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G10" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>25</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>12</v>
@@ -1059,11 +1099,14 @@
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G11" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>30</v>
       </c>
@@ -1083,11 +1126,14 @@
         <f t="shared" si="0"/>
         <v>13311.3</v>
       </c>
-      <c r="G12" s="13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G12" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>35</v>
       </c>
@@ -1107,16 +1153,19 @@
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G13" s="14" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G13" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>40</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>18</v>
@@ -1131,16 +1180,19 @@
         <f t="shared" si="0"/>
         <v>8469.75</v>
       </c>
-      <c r="G14" s="13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G14" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="H14" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>45</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>19</v>
@@ -1155,16 +1207,19 @@
         <f t="shared" si="0"/>
         <v>2493.48</v>
       </c>
-      <c r="G15" s="13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G15" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>50</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>20</v>
@@ -1179,11 +1234,14 @@
         <f t="shared" si="0"/>
         <v>7957.75</v>
       </c>
-      <c r="G16" s="14" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G16" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>55</v>
       </c>
@@ -1198,16 +1256,17 @@
       </c>
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
-      <c r="G17" s="25" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G17" s="38"/>
+      <c r="H17" s="25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>60</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>19</v>
@@ -1222,16 +1281,19 @@
         <f t="shared" si="0"/>
         <v>2493.48</v>
       </c>
-      <c r="G18" s="14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G18" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>65</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>20</v>
@@ -1246,16 +1308,19 @@
         <f t="shared" si="0"/>
         <v>7957.75</v>
       </c>
-      <c r="G19" s="14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G19" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>70</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>22</v>
@@ -1270,16 +1335,19 @@
         <f t="shared" si="0"/>
         <v>2493.48</v>
       </c>
-      <c r="G20" s="14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G20" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>22</v>
@@ -1294,19 +1362,22 @@
         <f t="shared" ref="F21" si="1">D21*E21</f>
         <v>2493.48</v>
       </c>
-      <c r="G21" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G21" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>75</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>24</v>
       </c>
       <c r="D22" s="4">
         <v>1</v>
@@ -1318,19 +1389,22 @@
         <f t="shared" si="0"/>
         <v>2525.98</v>
       </c>
-      <c r="G22" s="14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G22" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>80</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>25</v>
+      <c r="B23" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D23" s="4">
         <v>1</v>
@@ -1342,19 +1416,22 @@
         <f t="shared" si="0"/>
         <v>3205.31</v>
       </c>
-      <c r="G23" s="14" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G23" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>85</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>27</v>
+      <c r="B24" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D24" s="4">
         <v>1</v>
@@ -1366,19 +1443,22 @@
         <f t="shared" si="0"/>
         <v>2525.98</v>
       </c>
-      <c r="G24" s="14" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+      <c r="G24" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>90</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" s="4">
         <v>1</v>
@@ -1390,19 +1470,22 @@
         <f t="shared" si="0"/>
         <v>2525.98</v>
       </c>
-      <c r="G25" s="14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G25" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>95</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D26" s="4">
         <v>1</v>
@@ -1414,19 +1497,22 @@
         <f t="shared" si="0"/>
         <v>9927.32</v>
       </c>
-      <c r="G26" s="14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G26" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="4">
         <v>100</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D27" s="4">
         <v>1</v>
@@ -1438,19 +1524,22 @@
         <f t="shared" si="0"/>
         <v>9927.32</v>
       </c>
-      <c r="G27" s="14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G27" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>105</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
@@ -1462,41 +1551,49 @@
         <f t="shared" si="0"/>
         <v>2525.98</v>
       </c>
-      <c r="G28" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="28" x14ac:dyDescent="0.2">
-      <c r="A29" s="26">
+      <c r="G28" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="A29" s="4">
         <v>110</v>
       </c>
-      <c r="B29" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="C29" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D29" s="26">
-        <v>1</v>
-      </c>
-      <c r="E29" s="29">
+      <c r="B29" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1</v>
+      </c>
+      <c r="E29" s="7">
         <v>3135.92</v>
       </c>
-      <c r="F29" s="29">
+      <c r="F29" s="7">
         <f t="shared" si="0"/>
         <v>3135.92</v>
       </c>
-      <c r="G29" s="22"/>
-    </row>
-    <row r="30" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G29" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H29" s="21" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
         <v>115</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D30" s="4">
         <v>1</v>
@@ -1508,19 +1605,22 @@
         <f t="shared" si="0"/>
         <v>2525.98</v>
       </c>
-      <c r="G30" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G30" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
         <v>120</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D31" s="4">
         <v>1</v>
@@ -1532,19 +1632,22 @@
         <f t="shared" si="0"/>
         <v>5434.84</v>
       </c>
-      <c r="G31" s="14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G31" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="4">
         <v>125</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D32" s="4">
         <v>1</v>
@@ -1556,19 +1659,22 @@
         <f t="shared" si="0"/>
         <v>5434.84</v>
       </c>
-      <c r="G32" s="14" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+      <c r="G32" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A33" s="4">
         <v>130</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D33" s="4">
         <v>1</v>
@@ -1580,19 +1686,22 @@
         <f t="shared" si="0"/>
         <v>2576.7199999999998</v>
       </c>
-      <c r="G33" s="14" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+      <c r="G33" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H33" s="14" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A34" s="4">
         <v>135</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D34" s="4">
         <v>1</v>
@@ -1604,16 +1713,19 @@
         <f t="shared" si="0"/>
         <v>2355.16</v>
       </c>
-      <c r="G34" s="14" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G34" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="4">
         <v>140</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>12</v>
@@ -1628,19 +1740,22 @@
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G35" s="14" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G35" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="H35" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="4">
         <v>145</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D36" s="4">
         <v>1</v>
@@ -1652,41 +1767,47 @@
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G36" s="14" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="28" x14ac:dyDescent="0.2">
-      <c r="A37" s="26">
+      <c r="G36" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="A37" s="4">
         <v>150</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="26">
-        <v>1</v>
-      </c>
-      <c r="E37" s="29">
+      <c r="D37" s="4">
+        <v>1</v>
+      </c>
+      <c r="E37" s="7">
         <v>7602.17</v>
       </c>
-      <c r="F37" s="29">
+      <c r="F37" s="7">
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G37" s="22"/>
-    </row>
-    <row r="38" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G37" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H37" s="22"/>
+    </row>
+    <row r="38" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>155</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D38" s="4">
         <v>2</v>
@@ -1698,16 +1819,19 @@
         <f t="shared" si="0"/>
         <v>9524.76</v>
       </c>
-      <c r="G38" s="14" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G38" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="4">
         <v>160</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>14</v>
@@ -1722,19 +1846,22 @@
         <f t="shared" si="0"/>
         <v>6686.91</v>
       </c>
-      <c r="G39" s="21" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G39" s="36" t="s">
+        <v>123</v>
+      </c>
+      <c r="H39" s="21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A40" s="4">
         <v>165</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D40" s="4">
         <v>1</v>
@@ -1746,19 +1873,22 @@
         <f t="shared" si="0"/>
         <v>7602.17</v>
       </c>
-      <c r="G40" s="14" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G40" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="4">
         <v>170</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D41" s="4">
         <v>1</v>
@@ -1770,19 +1900,22 @@
         <f t="shared" si="0"/>
         <v>8025.57</v>
       </c>
-      <c r="G41" s="14" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G41" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="H41" s="14" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="4">
         <v>175</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D42" s="4">
         <v>1</v>
@@ -1794,17 +1927,18 @@
         <f t="shared" si="0"/>
         <v>51253.02</v>
       </c>
-      <c r="G42" s="6"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G42" s="37"/>
+      <c r="H42" s="6"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="4">
         <v>180</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D43" s="4">
         <v>99</v>
@@ -1816,17 +1950,18 @@
         <f t="shared" si="0"/>
         <v>10500.929999999998</v>
       </c>
-      <c r="G43" s="6"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G43" s="37"/>
+      <c r="H43" s="6"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="4">
         <v>185</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D44" s="4">
         <v>1</v>
@@ -1838,17 +1973,18 @@
         <f t="shared" si="0"/>
         <v>3404.7</v>
       </c>
-      <c r="G44" s="6"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G44" s="37"/>
+      <c r="H44" s="6"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="4">
         <v>190</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D45" s="4">
         <v>1</v>
@@ -1860,112 +1996,125 @@
         <f t="shared" si="0"/>
         <v>2054.6999999999998</v>
       </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G45" s="37"/>
+      <c r="H45" s="6"/>
+    </row>
+    <row r="46" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A46" s="19" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="7"/>
       <c r="F46" s="20"/>
-      <c r="G46" s="6"/>
-    </row>
-    <row r="47" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G46" s="39"/>
+      <c r="H46" s="6"/>
+    </row>
+    <row r="47" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A47" s="19" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="4"/>
       <c r="E47" s="7"/>
       <c r="F47" s="20"/>
-      <c r="G47" s="14" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="G47" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="H47" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="C48" s="38"/>
-      <c r="D48" s="38"/>
-      <c r="E48" s="38"/>
-      <c r="F48" s="39"/>
-      <c r="G48" s="38" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+      <c r="C48" s="32"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="H48" s="32" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C49" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F49" s="37">
+        <v>46</v>
+      </c>
+      <c r="F49" s="31">
         <f>SUM(F8:F48)-F42</f>
         <v>207277.30000000008</v>
       </c>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="E50" s="30" t="s">
-        <v>117</v>
+      <c r="G49" s="34"/>
+    </row>
+    <row r="50" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E50" s="26" t="s">
+        <v>104</v>
       </c>
       <c r="F50" s="10">
         <f>F49*0.08525</f>
         <v>17670.389825000009</v>
       </c>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="G50" s="34"/>
+    </row>
+    <row r="51" spans="3:8" x14ac:dyDescent="0.2">
       <c r="E51" s="9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F51" s="10">
         <f>F42</f>
         <v>51253.02</v>
       </c>
-    </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="G51" s="34"/>
+    </row>
+    <row r="52" spans="3:8" x14ac:dyDescent="0.2">
       <c r="E52" s="11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F52" s="12">
         <f>SUM(F8:F45)</f>
         <v>258530.32000000007</v>
       </c>
-      <c r="G52" s="31">
+      <c r="G52" s="35"/>
+      <c r="H52" s="27">
         <f>SUM(F49:F51)</f>
         <v>276200.70982500009</v>
       </c>
     </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="E53" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="G53" s="33">
-        <f>G52*0.1</f>
+    <row r="53" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E53" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="H53" s="28">
+        <f>H52*0.1</f>
         <v>27620.070982500009</v>
       </c>
     </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="E54" s="34" t="s">
-        <v>110</v>
-      </c>
-      <c r="F54" s="35"/>
-      <c r="G54" s="36">
-        <f>G52+G53</f>
+    <row r="54" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E54" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="F54" s="29"/>
+      <c r="G54" s="29"/>
+      <c r="H54" s="30">
+        <f>H52+H53</f>
         <v>303820.78080750012</v>
       </c>
     </row>

</xml_diff>

<commit_message>
A147-A160 into 3 windows
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64115B25-C962-1941-9B17-80836A94987F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998C48EC-F1DC-7545-83CE-BBFEB1590B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="660" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Window Estimate" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="130">
   <si>
     <t>Pella Window &amp; Door Replacement Estimate</t>
   </si>
@@ -444,6 +445,18 @@
   <si>
     <t>W 247-248
 (Kitchen east facing)</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>missing</t>
+  </si>
+  <si>
+    <t>Award</t>
+  </si>
+  <si>
+    <t>the upper bay window group at the central quadrant (photographs A-147 through A-160)</t>
   </si>
 </sst>
 </file>
@@ -655,8 +668,8 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -939,7 +952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -951,32 +964,32 @@
     <col min="8" max="8" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1002,7 +1015,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>10</v>
       </c>
@@ -1025,7 +1038,7 @@
       <c r="G8" s="20"/>
       <c r="H8" s="24"/>
     </row>
-    <row r="9" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>15</v>
       </c>
@@ -1051,8 +1064,11 @@
       <c r="H9" s="13" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>20</v>
       </c>
@@ -1078,8 +1094,11 @@
       <c r="H10" s="13" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>25</v>
       </c>
@@ -1105,8 +1124,11 @@
       <c r="H11" s="13" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>30</v>
       </c>
@@ -1132,8 +1154,11 @@
       <c r="H12" s="13" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>35</v>
       </c>
@@ -1160,7 +1185,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>40</v>
       </c>
@@ -1186,8 +1211,11 @@
       <c r="H14" s="13" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I14" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>45</v>
       </c>
@@ -1213,8 +1241,11 @@
       <c r="H15" s="13" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>50</v>
       </c>
@@ -1240,8 +1271,11 @@
       <c r="H16" s="14" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>55</v>
       </c>
@@ -1261,7 +1295,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>60</v>
       </c>
@@ -1288,7 +1322,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>65</v>
       </c>
@@ -1314,8 +1348,11 @@
       <c r="H19" s="14" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>70</v>
       </c>
@@ -1341,8 +1378,11 @@
       <c r="H20" s="14" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I20" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
         <v>68</v>
       </c>
@@ -1368,8 +1408,11 @@
       <c r="H21" s="14" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I21" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>75</v>
       </c>
@@ -1395,8 +1438,11 @@
       <c r="H22" s="14" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>80</v>
       </c>
@@ -1422,8 +1468,11 @@
       <c r="H23" s="14" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>85</v>
       </c>
@@ -1449,8 +1498,11 @@
       <c r="H24" s="14" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="I24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>90</v>
       </c>
@@ -1476,8 +1528,11 @@
       <c r="H25" s="14" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+      <c r="I25" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>95</v>
       </c>
@@ -1504,7 +1559,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="4">
         <v>100</v>
       </c>
@@ -1531,7 +1586,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>105</v>
       </c>
@@ -1558,7 +1613,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
         <v>110</v>
       </c>
@@ -1585,7 +1640,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
         <v>115</v>
       </c>
@@ -1612,7 +1667,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
         <v>120</v>
       </c>
@@ -1639,7 +1694,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="4">
         <v>125</v>
       </c>
@@ -2122,4 +2177,25 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D74D642-2015-4F42-A944-5629052DEDB0}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{1712afef-9f4e-4511-a60c-36df6704e051}" enabled="1" method="Standard" siteId="{4e9dbbfb-394a-4583-8810-53f81f819e3b}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Be more specific for "the kitchen corner windows (photographs A-184 through A-195)" -- A184 to A186 for east facing kitchen corner window; and A190 to A195 for north facing kitchen corner window
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998C48EC-F1DC-7545-83CE-BBFEB1590B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88AE55A-AADF-FD4D-99D0-3DDC3E700AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="660" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="130">
   <si>
     <t>Pella Window &amp; Door Replacement Estimate</t>
   </si>
@@ -456,7 +456,7 @@
     <t>Award</t>
   </si>
   <si>
-    <t>the upper bay window group at the central quadrant (photographs A-147 through A-160)</t>
+    <t>the four-season porch windows (photographs A-167 through A-175)</t>
   </si>
 </sst>
 </file>
@@ -1612,6 +1612,9 @@
       <c r="H28" s="14" t="s">
         <v>80</v>
       </c>
+      <c r="I28" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
@@ -1639,6 +1642,9 @@
       <c r="H29" s="21" t="s">
         <v>120</v>
       </c>
+      <c r="I29" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
@@ -1666,6 +1672,9 @@
       <c r="H30" s="14" t="s">
         <v>84</v>
       </c>
+      <c r="I30" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
@@ -1721,7 +1730,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A33" s="4">
         <v>130</v>
       </c>
@@ -1747,8 +1756,11 @@
       <c r="H33" s="14" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="I33" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A34" s="4">
         <v>135</v>
       </c>
@@ -1775,7 +1787,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="4">
         <v>140</v>
       </c>
@@ -1802,7 +1814,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="4">
         <v>145</v>
       </c>
@@ -1829,7 +1841,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>150</v>
       </c>
@@ -1854,7 +1866,7 @@
       </c>
       <c r="H37" s="22"/>
     </row>
-    <row r="38" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>155</v>
       </c>
@@ -1881,7 +1893,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="4">
         <v>160</v>
       </c>
@@ -1908,7 +1920,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A40" s="4">
         <v>165</v>
       </c>
@@ -1935,7 +1947,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="4">
         <v>170</v>
       </c>
@@ -1962,7 +1974,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="4">
         <v>175</v>
       </c>
@@ -1985,7 +1997,7 @@
       <c r="G42" s="37"/>
       <c r="H42" s="6"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="4">
         <v>180</v>
       </c>
@@ -2008,7 +2020,7 @@
       <c r="G43" s="37"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="4">
         <v>185</v>
       </c>
@@ -2031,7 +2043,7 @@
       <c r="G44" s="37"/>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="4">
         <v>190</v>
       </c>
@@ -2054,7 +2066,7 @@
       <c r="G45" s="37"/>
       <c r="H45" s="6"/>
     </row>
-    <row r="46" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A46" s="19" t="s">
         <v>68</v>
       </c>
@@ -2070,7 +2082,7 @@
       <c r="G46" s="39"/>
       <c r="H46" s="6"/>
     </row>
-    <row r="47" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A47" s="19" t="s">
         <v>68</v>
       </c>
@@ -2088,7 +2100,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="28" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
         <v>68</v>
       </c>

</xml_diff>

<commit_message>
Missing Upper window above main entry, A48 to A50
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88AE55A-AADF-FD4D-99D0-3DDC3E700AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0C80FF-60AC-D045-B479-AB3E697F3B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="660" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="130">
   <si>
     <t>Pella Window &amp; Door Replacement Estimate</t>
   </si>
@@ -366,10 +366,6 @@
     <t>Appraisal award</t>
   </si>
   <si>
-    <t>W 249-250
-(Kitchen east facung(</t>
-  </si>
-  <si>
     <t>A-185, 2.5.1</t>
   </si>
   <si>
@@ -456,7 +452,11 @@
     <t>Award</t>
   </si>
   <si>
-    <t>the four-season porch windows (photographs A-167 through A-175)</t>
+    <t>the kitchen corner windows (photographs A-184 through A-195)</t>
+  </si>
+  <si>
+    <t>W 249-250
+(Kitchen north facung(</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1009,7 @@
         <v>10</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>50</v>
@@ -1059,13 +1059,13 @@
         <v>7602.17</v>
       </c>
       <c r="G9" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1089,13 +1089,13 @@
         <v>7085.76</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>53</v>
       </c>
       <c r="I10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1119,13 +1119,13 @@
         <v>7602.17</v>
       </c>
       <c r="G11" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>54</v>
       </c>
       <c r="I11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1149,13 +1149,13 @@
         <v>13311.3</v>
       </c>
       <c r="G12" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>56</v>
       </c>
       <c r="I12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1179,7 +1179,7 @@
         <v>7602.17</v>
       </c>
       <c r="G13" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H13" s="14" t="s">
         <v>57</v>
@@ -1206,13 +1206,13 @@
         <v>8469.75</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>59</v>
       </c>
       <c r="I14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1236,13 +1236,13 @@
         <v>2493.48</v>
       </c>
       <c r="G15" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>60</v>
       </c>
       <c r="I15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1266,13 +1266,13 @@
         <v>7957.75</v>
       </c>
       <c r="G16" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1316,7 +1316,7 @@
         <v>2493.48</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H18" s="14" t="s">
         <v>65</v>
@@ -1343,13 +1343,13 @@
         <v>7957.75</v>
       </c>
       <c r="G19" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1373,13 +1373,13 @@
         <v>2493.48</v>
       </c>
       <c r="G20" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1403,13 +1403,13 @@
         <v>2493.48</v>
       </c>
       <c r="G21" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1417,7 +1417,7 @@
         <v>75</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>23</v>
@@ -1433,13 +1433,13 @@
         <v>2525.98</v>
       </c>
       <c r="G22" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -1447,7 +1447,7 @@
         <v>80</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>24</v>
@@ -1463,13 +1463,13 @@
         <v>3205.31</v>
       </c>
       <c r="G23" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H23" s="14" t="s">
         <v>72</v>
       </c>
       <c r="I23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -1477,7 +1477,7 @@
         <v>85</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>25</v>
@@ -1493,13 +1493,13 @@
         <v>2525.98</v>
       </c>
       <c r="G24" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="42" x14ac:dyDescent="0.2">
@@ -1523,13 +1523,13 @@
         <v>2525.98</v>
       </c>
       <c r="G25" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1553,7 +1553,7 @@
         <v>9927.32</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H26" s="14" t="s">
         <v>70</v>
@@ -1580,7 +1580,7 @@
         <v>9927.32</v>
       </c>
       <c r="G27" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H27" s="14" t="s">
         <v>79</v>
@@ -1607,13 +1607,13 @@
         <v>2525.98</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H28" s="14" t="s">
         <v>80</v>
       </c>
       <c r="I28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1637,13 +1637,13 @@
         <v>3135.92</v>
       </c>
       <c r="G29" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="H29" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="21" t="s">
-        <v>120</v>
-      </c>
       <c r="I29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1667,13 +1667,13 @@
         <v>2525.98</v>
       </c>
       <c r="G30" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H30" s="14" t="s">
         <v>84</v>
       </c>
       <c r="I30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
@@ -1697,10 +1697,13 @@
         <v>5434.84</v>
       </c>
       <c r="G31" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H31" s="14" t="s">
         <v>85</v>
+      </c>
+      <c r="I31" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
@@ -1724,10 +1727,10 @@
         <v>5434.84</v>
       </c>
       <c r="G32" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H32" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="42" x14ac:dyDescent="0.2">
@@ -1751,13 +1754,13 @@
         <v>2576.7199999999998</v>
       </c>
       <c r="G33" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H33" s="14" t="s">
         <v>73</v>
       </c>
       <c r="I33" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="42" x14ac:dyDescent="0.2">
@@ -1781,10 +1784,13 @@
         <v>2355.16</v>
       </c>
       <c r="G34" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H34" s="14" t="s">
         <v>74</v>
+      </c>
+      <c r="I34" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1808,7 +1814,7 @@
         <v>7602.17</v>
       </c>
       <c r="G35" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H35" s="14" t="s">
         <v>87</v>
@@ -1835,10 +1841,13 @@
         <v>7602.17</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
+      </c>
+      <c r="I36" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1862,7 +1871,7 @@
         <v>7602.17</v>
       </c>
       <c r="G37" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H37" s="22"/>
     </row>
@@ -1887,7 +1896,7 @@
         <v>9524.76</v>
       </c>
       <c r="G38" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H38" s="14" t="s">
         <v>90</v>
@@ -1914,7 +1923,7 @@
         <v>6686.91</v>
       </c>
       <c r="G39" s="36" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H39" s="21" t="s">
         <v>93</v>
@@ -1941,7 +1950,7 @@
         <v>7602.17</v>
       </c>
       <c r="G40" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H40" s="14" t="s">
         <v>94</v>
@@ -1968,7 +1977,7 @@
         <v>8025.57</v>
       </c>
       <c r="G41" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H41" s="14" t="s">
         <v>96</v>
@@ -2087,17 +2096,20 @@
         <v>68</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="4"/>
       <c r="E47" s="7"/>
       <c r="F47" s="20"/>
       <c r="G47" s="41" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="I47" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -2105,17 +2117,20 @@
         <v>68</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="C48" s="32"/>
       <c r="D48" s="32"/>
       <c r="E48" s="32"/>
       <c r="F48" s="33"/>
       <c r="G48" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H48" s="32" t="s">
-        <v>103</v>
+        <v>102</v>
+      </c>
+      <c r="I48" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="49" spans="3:8" x14ac:dyDescent="0.2">
@@ -2133,7 +2148,7 @@
     </row>
     <row r="50" spans="3:8" x14ac:dyDescent="0.2">
       <c r="E50" s="26" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F50" s="10">
         <f>F49*0.08525</f>
@@ -2198,7 +2213,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Missing UPPER SOUTHEAST FACING WINDOW AT FAMILY ROOM: A-106 and A-107. There is dent on A-107, right frame, several inches above the lower-right corner
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0C80FF-60AC-D045-B479-AB3E697F3B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA31BA12-3433-8C4A-968F-5DA4E26B6B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="660" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37940" yWindow="2040" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Window Estimate" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="131">
   <si>
     <t>Pella Window &amp; Door Replacement Estimate</t>
   </si>
@@ -209,9 +209,6 @@
 (Above living room)</t>
   </si>
   <si>
-    <t>A-54, A-55, A-56</t>
-  </si>
-  <si>
     <t>2 of the 3 sashes have new dents: A-39, A-40, A-41</t>
   </si>
   <si>
@@ -222,9 +219,6 @@
     <t>A-143, A-144</t>
   </si>
   <si>
-    <t>A-107</t>
-  </si>
-  <si>
     <t>Family W 229
 (upper south-east facing)</t>
   </si>
@@ -329,9 +323,6 @@
 (Garage)</t>
   </si>
   <si>
-    <t>2.8.1, 2.8.2, 2.8.3</t>
-  </si>
-  <si>
     <t>South W 375-377
 (Upper-top)</t>
   </si>
@@ -452,11 +443,23 @@
     <t>Award</t>
   </si>
   <si>
-    <t>the kitchen corner windows (photographs A-184 through A-195)</t>
-  </si>
-  <si>
     <t>W 249-250
 (Kitchen north facung(</t>
+  </si>
+  <si>
+    <t>2.8.1, 2.8.2, 2.8.3, A-216</t>
+  </si>
+  <si>
+    <t>added</t>
+  </si>
+  <si>
+    <t>A-54, A-55, A-56, 1.5.1, 1.5.2.1, 1.5.2.2, 1.5.3, 1.5.4</t>
+  </si>
+  <si>
+    <t>UPPER SOUTHEAST FACING WINDOW AT FAMILY ROOM</t>
+  </si>
+  <si>
+    <t>A-107, 2.1.1</t>
   </si>
 </sst>
 </file>
@@ -952,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -964,32 +967,32 @@
     <col min="8" max="8" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1009,13 +1012,13 @@
         <v>10</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>10</v>
       </c>
@@ -1038,7 +1041,7 @@
       <c r="G8" s="20"/>
       <c r="H8" s="24"/>
     </row>
-    <row r="9" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>15</v>
       </c>
@@ -1059,16 +1062,16 @@
         <v>7602.17</v>
       </c>
       <c r="G9" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>52</v>
       </c>
       <c r="I9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>20</v>
       </c>
@@ -1089,16 +1092,19 @@
         <v>7085.76</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>53</v>
       </c>
       <c r="I10" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+      <c r="J10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>25</v>
       </c>
@@ -1119,16 +1125,16 @@
         <v>7602.17</v>
       </c>
       <c r="G11" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>54</v>
       </c>
       <c r="I11" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>30</v>
       </c>
@@ -1149,16 +1155,19 @@
         <v>13311.3</v>
       </c>
       <c r="G12" s="36" t="s">
-        <v>105</v>
-      </c>
-      <c r="H12" s="13" t="s">
-        <v>56</v>
+        <v>102</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>128</v>
       </c>
       <c r="I12" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+      <c r="J12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>35</v>
       </c>
@@ -1179,18 +1188,18 @@
         <v>7602.17</v>
       </c>
       <c r="G13" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>40</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>18</v>
@@ -1206,21 +1215,21 @@
         <v>8469.75</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I14" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>45</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>19</v>
@@ -1236,21 +1245,21 @@
         <v>2493.48</v>
       </c>
       <c r="G15" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="I15" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>50</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>20</v>
@@ -1266,13 +1275,13 @@
         <v>7957.75</v>
       </c>
       <c r="G16" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I16" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1292,7 +1301,7 @@
       <c r="F17" s="18"/>
       <c r="G17" s="38"/>
       <c r="H17" s="25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1300,7 +1309,7 @@
         <v>60</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>19</v>
@@ -1316,10 +1325,10 @@
         <v>2493.48</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1327,7 +1336,7 @@
         <v>65</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>20</v>
@@ -1343,13 +1352,13 @@
         <v>7957.75</v>
       </c>
       <c r="G19" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I19" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1357,7 +1366,7 @@
         <v>70</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>22</v>
@@ -1373,21 +1382,21 @@
         <v>2493.48</v>
       </c>
       <c r="G20" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I20" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>22</v>
@@ -1403,13 +1412,13 @@
         <v>2493.48</v>
       </c>
       <c r="G21" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I21" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1417,7 +1426,7 @@
         <v>75</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>23</v>
@@ -1433,13 +1442,13 @@
         <v>2525.98</v>
       </c>
       <c r="G22" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I22" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -1447,7 +1456,7 @@
         <v>80</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>24</v>
@@ -1463,13 +1472,13 @@
         <v>3205.31</v>
       </c>
       <c r="G23" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -1477,7 +1486,7 @@
         <v>85</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>25</v>
@@ -1493,13 +1502,13 @@
         <v>2525.98</v>
       </c>
       <c r="G24" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I24" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="42" x14ac:dyDescent="0.2">
@@ -1507,7 +1516,7 @@
         <v>90</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>23</v>
@@ -1523,13 +1532,13 @@
         <v>2525.98</v>
       </c>
       <c r="G25" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I25" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1537,7 +1546,7 @@
         <v>95</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>26</v>
@@ -1553,10 +1562,13 @@
         <v>9927.32</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
+      </c>
+      <c r="I26" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1564,7 +1576,7 @@
         <v>100</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>26</v>
@@ -1580,10 +1592,10 @@
         <v>9927.32</v>
       </c>
       <c r="G27" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1591,7 +1603,7 @@
         <v>105</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>23</v>
@@ -1607,13 +1619,13 @@
         <v>2525.98</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1621,7 +1633,7 @@
         <v>110</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>27</v>
@@ -1637,13 +1649,13 @@
         <v>3135.92</v>
       </c>
       <c r="G29" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H29" s="21" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I29" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1651,7 +1663,7 @@
         <v>115</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>25</v>
@@ -1667,13 +1679,13 @@
         <v>2525.98</v>
       </c>
       <c r="G30" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I30" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
@@ -1697,13 +1709,13 @@
         <v>5434.84</v>
       </c>
       <c r="G31" s="36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I31" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
@@ -1727,10 +1739,10 @@
         <v>5434.84</v>
       </c>
       <c r="G32" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H32" s="14" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="42" x14ac:dyDescent="0.2">
@@ -1738,7 +1750,7 @@
         <v>130</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>31</v>
@@ -1754,13 +1766,13 @@
         <v>2576.7199999999998</v>
       </c>
       <c r="G33" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I33" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="42" x14ac:dyDescent="0.2">
@@ -1768,7 +1780,7 @@
         <v>135</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>32</v>
@@ -1784,13 +1796,13 @@
         <v>2355.16</v>
       </c>
       <c r="G34" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I34" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1798,7 +1810,7 @@
         <v>140</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>12</v>
@@ -1814,10 +1826,10 @@
         <v>7602.17</v>
       </c>
       <c r="G35" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
@@ -1841,13 +1853,13 @@
         <v>7602.17</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I36" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1855,7 +1867,7 @@
         <v>150</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>12</v>
@@ -1871,7 +1883,7 @@
         <v>7602.17</v>
       </c>
       <c r="G37" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H37" s="22"/>
     </row>
@@ -1880,7 +1892,7 @@
         <v>155</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>35</v>
@@ -1896,10 +1908,13 @@
         <v>9524.76</v>
       </c>
       <c r="G38" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>90</v>
+        <v>126</v>
+      </c>
+      <c r="I38" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1907,7 +1922,7 @@
         <v>160</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>14</v>
@@ -1923,10 +1938,10 @@
         <v>6686.91</v>
       </c>
       <c r="G39" s="36" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H39" s="21" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1934,7 +1949,7 @@
         <v>165</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>34</v>
@@ -1950,10 +1965,10 @@
         <v>7602.17</v>
       </c>
       <c r="G40" s="36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -1961,7 +1976,7 @@
         <v>170</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>36</v>
@@ -1977,10 +1992,13 @@
         <v>8025.57</v>
       </c>
       <c r="G41" s="36" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>96</v>
+        <v>93</v>
+      </c>
+      <c r="I41" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
@@ -2077,13 +2095,13 @@
     </row>
     <row r="46" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A46" s="19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="7"/>
@@ -2093,44 +2111,44 @@
     </row>
     <row r="47" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A47" s="19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="4"/>
       <c r="E47" s="7"/>
       <c r="F47" s="20"/>
       <c r="G47" s="41" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I47" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C48" s="32"/>
       <c r="D48" s="32"/>
       <c r="E48" s="32"/>
       <c r="F48" s="33"/>
       <c r="G48" s="40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H48" s="32" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I48" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="3:8" x14ac:dyDescent="0.2">
@@ -2148,7 +2166,7 @@
     </row>
     <row r="50" spans="3:8" x14ac:dyDescent="0.2">
       <c r="E50" s="26" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F50" s="10">
         <f>F49*0.08525</f>
@@ -2182,7 +2200,7 @@
     </row>
     <row r="53" spans="3:8" x14ac:dyDescent="0.2">
       <c r="E53" s="26" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H53" s="28">
         <f>H52*0.1</f>
@@ -2191,7 +2209,7 @@
     </row>
     <row r="54" spans="3:8" x14ac:dyDescent="0.2">
       <c r="E54" s="11" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F54" s="29"/>
       <c r="G54" s="29"/>
@@ -2213,7 +2231,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated docs from 19+ windows to 25+ windows
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA31BA12-3433-8C4A-968F-5DA4E26B6B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD9A8CD-9A3D-DD47-80E2-57D66963FE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="37940" yWindow="2040" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="133">
   <si>
     <t>Pella Window &amp; Door Replacement Estimate</t>
   </si>
@@ -460,6 +460,12 @@
   </si>
   <si>
     <t>A-107, 2.1.1</t>
+  </si>
+  <si>
+    <t>Already in a sliding door 49(b)</t>
+  </si>
+  <si>
+    <t>Need to confirm?</t>
   </si>
 </sst>
 </file>
@@ -1251,7 +1257,10 @@
         <v>130</v>
       </c>
       <c r="I15" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+      <c r="J15" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="28" x14ac:dyDescent="0.2">
@@ -1284,7 +1293,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>55</v>
       </c>
@@ -1304,7 +1313,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>60</v>
       </c>
@@ -1331,7 +1340,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>65</v>
       </c>
@@ -1361,7 +1370,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>70</v>
       </c>
@@ -1391,7 +1400,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
         <v>66</v>
       </c>
@@ -1421,7 +1430,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>75</v>
       </c>
@@ -1451,7 +1460,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>80</v>
       </c>
@@ -1481,7 +1490,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>85</v>
       </c>
@@ -1511,7 +1520,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="42" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="42" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>90</v>
       </c>
@@ -1541,7 +1550,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>95</v>
       </c>
@@ -1570,8 +1579,11 @@
       <c r="I26" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+      <c r="J26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="4">
         <v>100</v>
       </c>
@@ -1598,7 +1610,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>105</v>
       </c>
@@ -1628,7 +1640,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
         <v>110</v>
       </c>
@@ -1658,7 +1670,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
         <v>115</v>
       </c>
@@ -1688,7 +1700,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
         <v>120</v>
       </c>
@@ -1718,7 +1730,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="4">
         <v>125</v>
       </c>
@@ -1745,7 +1757,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="42" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="42" x14ac:dyDescent="0.2">
       <c r="A33" s="4">
         <v>130</v>
       </c>
@@ -1775,7 +1787,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="42" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="42" x14ac:dyDescent="0.2">
       <c r="A34" s="4">
         <v>135</v>
       </c>
@@ -1805,7 +1817,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="4">
         <v>140</v>
       </c>
@@ -1832,7 +1844,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="4">
         <v>145</v>
       </c>
@@ -1862,7 +1874,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>150</v>
       </c>
@@ -1887,7 +1899,7 @@
       </c>
       <c r="H37" s="22"/>
     </row>
-    <row r="38" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>155</v>
       </c>
@@ -1917,7 +1929,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="4">
         <v>160</v>
       </c>
@@ -1944,7 +1956,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A40" s="4">
         <v>165</v>
       </c>
@@ -1971,7 +1983,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="4">
         <v>170</v>
       </c>
@@ -2000,8 +2012,11 @@
       <c r="I41" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="4">
         <v>175</v>
       </c>
@@ -2024,7 +2039,7 @@
       <c r="G42" s="37"/>
       <c r="H42" s="6"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="4">
         <v>180</v>
       </c>
@@ -2047,7 +2062,7 @@
       <c r="G43" s="37"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="4">
         <v>185</v>
       </c>
@@ -2070,7 +2085,7 @@
       <c r="G44" s="37"/>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="4">
         <v>190</v>
       </c>
@@ -2093,7 +2108,7 @@
       <c r="G45" s="37"/>
       <c r="H45" s="6"/>
     </row>
-    <row r="46" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A46" s="19" t="s">
         <v>66</v>
       </c>
@@ -2109,7 +2124,7 @@
       <c r="G46" s="39"/>
       <c r="H46" s="6"/>
     </row>
-    <row r="47" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A47" s="19" t="s">
         <v>66</v>
       </c>
@@ -2130,7 +2145,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
         <v>66</v>
       </c>

</xml_diff>

<commit_message>
Receipt of mailing the motion notice and redacted complaint
</commit_message>
<xml_diff>
--- a/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
+++ b/EventDocuments/CommunicationWithPureConstruction/Window_Replacement_Estimate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/EventDocuments/CommunicationWithPureConstruction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD9A8CD-9A3D-DD47-80E2-57D66963FE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82F73C9-4AAA-0043-922A-78EAF0E1791C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37940" yWindow="2040" windowWidth="31720" windowHeight="19800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1520" yWindow="660" windowWidth="31720" windowHeight="19800" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Window Estimate" sheetId="1" r:id="rId1"/>
@@ -456,9 +456,6 @@
     <t>A-54, A-55, A-56, 1.5.1, 1.5.2.1, 1.5.2.2, 1.5.3, 1.5.4</t>
   </si>
   <si>
-    <t>UPPER SOUTHEAST FACING WINDOW AT FAMILY ROOM</t>
-  </si>
-  <si>
     <t>A-107, 2.1.1</t>
   </si>
   <si>
@@ -466,6 +463,9 @@
   </si>
   <si>
     <t>Need to confirm?</t>
+  </si>
+  <si>
+    <t>Minnesota Department of Commerce</t>
   </si>
 </sst>
 </file>
@@ -1254,7 +1254,7 @@
         <v>102</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I15" t="s">
         <v>122</v>
@@ -1580,7 +1580,7 @@
         <v>123</v>
       </c>
       <c r="J26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="28" x14ac:dyDescent="0.2">
@@ -2013,7 +2013,7 @@
         <v>66</v>
       </c>
       <c r="J41" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
@@ -2241,12 +2241,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D74D642-2015-4F42-A944-5629052DEDB0}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>129</v>
+        <v>132</v>
+      </c>
+      <c r="E1">
+        <f>17*6400</f>
+        <v>108800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>